<commit_message>
update excel importing logic, crm-translate
</commit_message>
<xml_diff>
--- a/crystal-backend/docs/samples/crm-customers-sample.xlsx
+++ b/crystal-backend/docs/samples/crm-customers-sample.xlsx
@@ -36,14 +36,14 @@
     <comment ref="C1" authorId="0">
       <text>
         <r>
-          <t>The customer's user_pk in the user management system (PLATFORM, a number). Kept as an unverified identifier.</t>
+          <t>The customer's user_pk in the user management system (a number). Kept as an unverified identifier.</t>
         </r>
       </text>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>The customer's user_id (login) in the user management system (PLATFORM). Kept as an unverified identifier.</t>
+          <t>The customer's user_id (login) in the user management system. Kept as an unverified identifier.</t>
         </r>
       </text>
     </comment>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="105">
   <si>
     <t>E-shop PK *</t>
   </si>
@@ -290,12 +290,12 @@
     <t>Farmer</t>
   </si>
   <si>
+    <t>Scientist</t>
+  </si>
+  <si>
     <t>Teacher</t>
   </si>
   <si>
-    <t>Scientist</t>
-  </si>
-  <si>
     <t>Engineer</t>
   </si>
   <si>
@@ -323,48 +323,6 @@
     <t>Other</t>
   </si>
   <si>
-    <t>Account director</t>
-  </si>
-  <si>
-    <t>Accountant</t>
-  </si>
-  <si>
-    <t>CEO</t>
-  </si>
-  <si>
-    <t>Chairman</t>
-  </si>
-  <si>
-    <t>Designer</t>
-  </si>
-  <si>
-    <t>Head of IT</t>
-  </si>
-  <si>
-    <t>IT manager</t>
-  </si>
-  <si>
-    <t>Nurse</t>
-  </si>
-  <si>
-    <t>Procurement lead</t>
-  </si>
-  <si>
-    <t>Sales manager</t>
-  </si>
-  <si>
-    <t>Software engineer</t>
-  </si>
-  <si>
-    <t>Store manager</t>
-  </si>
-  <si>
-    <t>Store operations</t>
-  </si>
-  <si>
-    <t>Workshop lead</t>
-  </si>
-  <si>
     <t>Location</t>
   </si>
   <si>
@@ -386,25 +344,16 @@
     <t>06</t>
   </si>
   <si>
-    <t>14</t>
+    <t>4</t>
   </si>
   <si>
     <t>East Province</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>04</t>
   </si>
   <si>
-    <t>1102</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>11</t>
+    <t>7</t>
   </si>
   <si>
     <t>Highland Region</t>
@@ -413,103 +362,46 @@
     <t>07</t>
   </si>
   <si>
-    <t>12</t>
+    <t>2</t>
   </si>
   <si>
     <t>North Province</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>02</t>
   </si>
   <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>13</t>
+    <t>3</t>
   </si>
   <si>
     <t>South Province</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>03</t>
   </si>
   <si>
-    <t>1101</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>1103</t>
+    <t>5</t>
   </si>
   <si>
     <t>West Province</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>05</t>
   </si>
   <si>
     <t>Project</t>
   </si>
   <si>
-    <t>PLATFORM</t>
-  </si>
-  <si>
-    <t>Vendor platform (PID)</t>
-  </si>
-  <si>
-    <t>CRYSTAL</t>
-  </si>
-  <si>
-    <t>Crystal web and console</t>
-  </si>
-  <si>
-    <t>EPRODUCT</t>
-  </si>
-  <si>
-    <t>Eproduct site and agencies</t>
-  </si>
-  <si>
-    <t>ESHOP</t>
-  </si>
-  <si>
-    <t>Eshop</t>
-  </si>
-  <si>
-    <t>APPSTORE</t>
-  </si>
-  <si>
-    <t>Appstore</t>
-  </si>
-  <si>
-    <t>KARAOKE</t>
-  </si>
-  <si>
-    <t>Karaoke licence service</t>
-  </si>
-  <si>
-    <t>CRM1</t>
-  </si>
-  <si>
-    <t>CRM</t>
+    <t>USER_MANAGER</t>
+  </si>
+  <si>
+    <t>User ID Management System</t>
+  </si>
+  <si>
+    <t>E_SHOP</t>
+  </si>
+  <si>
+    <t>E_shop</t>
   </si>
 </sst>
 </file>
@@ -982,7 +874,7 @@
         <v>19</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1017,7 +909,7 @@
         <v>26</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1052,7 +944,7 @@
         <v>32</v>
       </c>
       <c r="K4">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1087,7 +979,7 @@
         <v>38</v>
       </c>
       <c r="K5">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1122,7 +1014,7 @@
         <v>44</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1157,7 +1049,7 @@
         <v>50</v>
       </c>
       <c r="K7">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1227,7 +1119,7 @@
         <v>62</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="6:12" x14ac:dyDescent="0.25"/>
@@ -2231,22 +2123,22 @@
       <formula1>"M,F"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Location ID" error="Choose an ID from the Locations sheet" sqref="I10:I1001">
-      <formula1>'Locations'!$A$2:$A$16</formula1>
+      <formula1>'Locations'!$A$2:$A$8</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Location ID" error="Choose an ID from the Locations sheet" sqref="I2:I1001">
-      <formula1>'Locations'!$A$2:$A$16</formula1>
+      <formula1>'Locations'!$A$2:$A$8</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Job title ID" error="Choose an ID from the Job titles sheet" sqref="K10:K1001">
-      <formula1>'Job titles'!$A$2:$A$28</formula1>
+      <formula1>'Job titles'!$A$2:$A$14</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Job title ID" error="Choose an ID from the Job titles sheet" sqref="K2:K1001">
-      <formula1>'Job titles'!$A$2:$A$28</formula1>
+      <formula1>'Job titles'!$A$2:$A$14</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Origin project" error="Choose a code from the Projects sheet, or leave it empty" sqref="L10:L1001">
-      <formula1>'Projects'!$A$2:$A$8</formula1>
+      <formula1>'Projects'!$A$2:$A$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Origin project" error="Choose a code from the Projects sheet, or leave it empty" sqref="L2:L1001">
-      <formula1>'Projects'!$A$2:$A$8</formula1>
+      <formula1>'Projects'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2257,7 +2149,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2282,7 +2174,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>66</v>
@@ -2290,7 +2182,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>67</v>
@@ -2298,7 +2190,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>68</v>
@@ -2306,7 +2198,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>69</v>
@@ -2314,7 +2206,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
         <v>70</v>
@@ -2322,7 +2214,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
@@ -2330,7 +2222,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
         <v>72</v>
@@ -2338,7 +2230,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>73</v>
@@ -2346,7 +2238,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>74</v>
@@ -2354,7 +2246,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>75</v>
@@ -2362,7 +2254,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>76</v>
@@ -2370,122 +2262,10 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2496,7 +2276,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2509,10 +2289,10 @@
         <v>63</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2520,164 +2300,76 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>110</v>
-      </c>
-      <c r="B9" t="s">
-        <v>109</v>
-      </c>
-      <c r="C9" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>112</v>
-      </c>
-      <c r="B10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>114</v>
-      </c>
-      <c r="B11" t="s">
-        <v>115</v>
-      </c>
-      <c r="C11" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>116</v>
-      </c>
-      <c r="B12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>118</v>
-      </c>
-      <c r="B13" t="s">
-        <v>115</v>
-      </c>
-      <c r="C13" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>120</v>
-      </c>
-      <c r="B14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C14" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B15" t="s">
-        <v>121</v>
-      </c>
-      <c r="C15" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>124</v>
-      </c>
-      <c r="B16" t="s">
-        <v>121</v>
-      </c>
-      <c r="C16" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2688,7 +2380,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2698,90 +2390,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>101</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>